<commit_message>
Update tile URLs in configuration files to use 'dark_nolabels' instead of 'dark_all'. Modify setup.sh to enhance sudo permissions for the service helper, ensuring proper functionality checks. Adjust fetch_tiles.py and related scripts to reflect the new tile URL. Improve CSS styles for dark theme elements and update JavaScript to handle service state display more effectively.
</commit_message>
<xml_diff>
--- a/Example Docs/Newsnation Global Path Naming.xlsx
+++ b/Example Docs/Newsnation Global Path Naming.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nexstartv.sharepoint.com/teams/NewsNationEngineering/Shared Documents/General/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26CA7F966D4A52C6/Code/NexNOC/Example Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2897" documentId="14_{AA77E42B-1188-4023-99CE-412A287F8599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB63D4F4-4CF4-4E0A-94B3-80DA578BDFD7}"/>
+  <xr:revisionPtr revIDLastSave="2898" documentId="14_{AA77E42B-1188-4023-99CE-412A287F8599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF44593C-D8D5-49FA-81CF-072765EEB763}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="1635" windowWidth="23235" windowHeight="11355" tabRatio="816" firstSheet="11" activeTab="11" xr2:uid="{98E875BD-AF76-45D8-B210-E932B4556ABF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" tabRatio="816" activeTab="1" xr2:uid="{98E875BD-AF76-45D8-B210-E932B4556ABF}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover Page" sheetId="4" r:id="rId1"/>
@@ -3390,7 +3390,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="15">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3906,15 +3906,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3951,6 +3942,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3966,17 +3963,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -3991,7 +3982,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -4333,7 +4333,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E6FE14C-CA21-486E-B817-8C185D5E3288}" name="Table1" displayName="Table1" ref="A1:AA103" totalsRowShown="0" headerRowDxfId="59" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:AA103" xr:uid="{1E6FE14C-CA21-486E-B817-8C185D5E3288}"/>
+  <autoFilter ref="A1:AA103" xr:uid="{1E6FE14C-CA21-486E-B817-8C185D5E3288}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="WDCW"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AA90">
     <sortCondition ref="A1:A90"/>
   </sortState>
@@ -4610,9 +4616,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4650,7 +4656,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -4756,7 +4762,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4898,7 +4904,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -4907,7 +4913,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{442FA5C4-1D90-4B30-A8FD-EB559BAA41D8}">
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.125" bestFit="1" customWidth="1"/>
@@ -4917,67 +4923,67 @@
     <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="19.149999999999999">
-      <c r="A1" s="47" t="s">
+    <row r="1" spans="1:6" ht="19.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="49"/>
-    </row>
-    <row r="2" spans="1:6" ht="19.149999999999999">
-      <c r="A2" s="50" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="46"/>
+    </row>
+    <row r="2" spans="1:6" ht="19.5" x14ac:dyDescent="0.2">
+      <c r="A2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="C2" s="51"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="52"/>
-    </row>
-    <row r="3" spans="1:6" ht="19.149999999999999">
-      <c r="A3" s="53" t="s">
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="49"/>
+    </row>
+    <row r="3" spans="1:6" ht="19.5" x14ac:dyDescent="0.2">
+      <c r="A3" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="55"/>
-    </row>
-    <row r="4" spans="1:6" ht="44.25" customHeight="1">
-      <c r="A4" s="56" t="s">
+      <c r="B3" s="51"/>
+      <c r="C3" s="51"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="51"/>
+      <c r="F3" s="52"/>
+    </row>
+    <row r="4" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="57"/>
-      <c r="C4" s="57"/>
-      <c r="D4" s="57"/>
-      <c r="E4" s="57"/>
-      <c r="F4" s="58"/>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="44" t="s">
+      <c r="B4" s="54"/>
+      <c r="C4" s="54"/>
+      <c r="D4" s="54"/>
+      <c r="E4" s="54"/>
+      <c r="F4" s="55"/>
+    </row>
+    <row r="5" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="56" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="59"/>
-      <c r="E5" s="62" t="s">
+      <c r="B5" s="57"/>
+      <c r="C5" s="57"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="61" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="63"/>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="F5" s="62"/>
+    </row>
+    <row r="6" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="45"/>
-      <c r="D6" s="60"/>
+      <c r="C6" s="57"/>
+      <c r="D6" s="59"/>
       <c r="E6" s="8" t="s">
         <v>6</v>
       </c>
@@ -4985,15 +4991,15 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="45" t="s">
+      <c r="B7" s="57" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="45"/>
-      <c r="D7" s="60"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="59"/>
       <c r="E7" s="2" t="s">
         <v>9</v>
       </c>
@@ -5001,15 +5007,15 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="45" t="s">
+      <c r="B8" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="45"/>
-      <c r="D8" s="60"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="59"/>
       <c r="E8" s="2" t="s">
         <v>12</v>
       </c>
@@ -5017,15 +5023,15 @@
         <v>14</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="45" t="s">
+      <c r="B9" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="45"/>
-      <c r="D9" s="60"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="59"/>
       <c r="E9" s="2" t="s">
         <v>15</v>
       </c>
@@ -5033,15 +5039,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="45" t="s">
+      <c r="B10" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="45"/>
-      <c r="D10" s="60"/>
+      <c r="C10" s="57"/>
+      <c r="D10" s="59"/>
       <c r="E10" s="2" t="s">
         <v>18</v>
       </c>
@@ -5049,15 +5055,15 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="57" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="45"/>
-      <c r="D11" s="60"/>
+      <c r="C11" s="57"/>
+      <c r="D11" s="59"/>
       <c r="E11" s="2" t="s">
         <v>21</v>
       </c>
@@ -5065,15 +5071,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="45" t="s">
+      <c r="B12" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="45"/>
-      <c r="D12" s="60"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="59"/>
       <c r="E12" s="2" t="s">
         <v>24</v>
       </c>
@@ -5081,15 +5087,15 @@
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" ht="15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="45" t="s">
+      <c r="B13" s="57" t="s">
         <v>11</v>
       </c>
-      <c r="C13" s="45"/>
-      <c r="D13" s="61"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="60"/>
       <c r="E13" s="2" t="s">
         <v>25</v>
       </c>
@@ -5097,21 +5103,21 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="44" t="s">
+    <row r="14" spans="1:6" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="56" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="45"/>
-      <c r="C14" s="45" t="s">
+      <c r="B14" s="57"/>
+      <c r="C14" s="57" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45" t="s">
+      <c r="D14" s="57"/>
+      <c r="E14" s="57" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="46"/>
-    </row>
-    <row r="15" spans="1:6" ht="14.45" thickBot="1">
+      <c r="F14" s="63"/>
+    </row>
+    <row r="15" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
@@ -5131,11 +5137,20 @@
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
@@ -5145,15 +5160,6 @@
     <mergeCell ref="E5:F5"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
@@ -5164,7 +5170,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEEF543F-629A-409B-9B5F-BC96E46FA491}">
   <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.875" customWidth="1"/>
     <col min="2" max="2" width="12.5" customWidth="1"/>
@@ -5178,7 +5184,7 @@
     <col min="10" max="10" width="80.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="24" customFormat="1" ht="14.25" customHeight="1">
+    <row r="1" spans="1:10" s="24" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>938</v>
       </c>
@@ -5210,7 +5216,7 @@
         <v>947</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25" customHeight="1">
+    <row r="2" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>948</v>
       </c>
@@ -5233,7 +5239,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25" customHeight="1">
+    <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>955</v>
       </c>
@@ -5262,7 +5268,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25" customHeight="1">
+    <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>955</v>
       </c>
@@ -5288,12 +5294,12 @@
         <v>966</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="14.25" customHeight="1">
+    <row r="5" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="J5" t="s">
         <v>967</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.25" customHeight="1">
+    <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>948</v>
       </c>
@@ -5316,7 +5322,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.25" customHeight="1">
+    <row r="7" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>955</v>
       </c>
@@ -5342,7 +5348,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="14.25" customHeight="1">
+    <row r="8" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>955</v>
       </c>
@@ -5365,7 +5371,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="14.25" customHeight="1">
+    <row r="10" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>955</v>
       </c>
@@ -5391,7 +5397,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.25" customHeight="1">
+    <row r="12" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>955</v>
       </c>
@@ -5417,7 +5423,7 @@
         <v>989</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="14.25" customHeight="1">
+    <row r="13" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>955</v>
       </c>
@@ -5443,7 +5449,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="14.25" customHeight="1">
+    <row r="15" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>948</v>
       </c>
@@ -5469,7 +5475,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="14.25" customHeight="1">
+    <row r="16" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
         <v>1001</v>
       </c>
@@ -5483,7 +5489,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="14.25" customHeight="1">
+    <row r="18" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>948</v>
       </c>
@@ -5509,7 +5515,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="14.25" customHeight="1">
+    <row r="19" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>1012</v>
       </c>
@@ -5523,7 +5529,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="14.25" customHeight="1">
+    <row r="21" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>1016</v>
       </c>
@@ -5549,7 +5555,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="14.25" customHeight="1">
+    <row r="23" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>948</v>
       </c>
@@ -5572,7 +5578,7 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="14.25" customHeight="1">
+    <row r="24" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
         <v>1029</v>
       </c>
@@ -5586,7 +5592,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="14.25" customHeight="1">
+    <row r="26" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>948</v>
       </c>
@@ -5615,7 +5621,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="14.25" customHeight="1">
+    <row r="27" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D27" t="s">
         <v>1038</v>
       </c>
@@ -5626,7 +5632,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="14.25" customHeight="1">
+    <row r="29" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1016</v>
       </c>
@@ -5652,7 +5658,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="14.25" customHeight="1">
+    <row r="32" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>948</v>
       </c>
@@ -5660,7 +5666,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="33" spans="1:9" ht="14.25" customHeight="1">
+    <row r="33" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>948</v>
       </c>
@@ -5671,7 +5677,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="14.25" customHeight="1">
+    <row r="34" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>948</v>
       </c>
@@ -5682,7 +5688,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="36" spans="1:9" ht="14.25" customHeight="1">
+    <row r="36" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>1048</v>
       </c>
@@ -5693,7 +5699,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="14.25" customHeight="1">
+    <row r="38" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>955</v>
       </c>
@@ -5707,7 +5713,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="14.25" customHeight="1">
+    <row r="39" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>955</v>
       </c>
@@ -5721,7 +5727,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="14.25" customHeight="1">
+    <row r="40" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>955</v>
       </c>
@@ -5744,7 +5750,7 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5544A448-34A5-4C53-8435-81CC687B7CCF}">
   <dimension ref="A1:AA45"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.125" customWidth="1"/>
     <col min="2" max="2" width="16" style="36" bestFit="1" customWidth="1"/>
@@ -5765,7 +5771,7 @@
     <col min="28" max="28" width="21.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="24" customFormat="1">
+    <row r="1" spans="1:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>32</v>
       </c>
@@ -5848,7 +5854,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:27">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="B2" t="s">
         <v>1050</v>
       </c>
@@ -5865,7 +5871,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1054</v>
       </c>
@@ -5885,7 +5891,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1057</v>
       </c>
@@ -5905,7 +5911,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1060</v>
       </c>
@@ -5925,7 +5931,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="6" spans="1:27">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1063</v>
       </c>
@@ -5945,7 +5951,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1066</v>
       </c>
@@ -5965,7 +5971,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1069</v>
       </c>
@@ -5985,8 +5991,8 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="24" ht="13.5" customHeight="1"/>
-    <row r="45" ht="15" customHeight="1"/>
+    <row r="24" ht="13.5" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0"/>
   <printOptions gridLines="1"/>
@@ -6001,7 +6007,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C817F748-9FC0-4945-8E6C-495F2D507CFC}">
   <dimension ref="A2:K6"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.875" customWidth="1"/>
     <col min="2" max="3" width="17.625" customWidth="1"/>
@@ -6015,7 +6021,7 @@
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="42" t="s">
         <v>32</v>
       </c>
@@ -6050,7 +6056,7 @@
         <v>1075</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="14.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1076</v>
       </c>
@@ -6085,7 +6091,7 @@
         <v>1083</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1084</v>
       </c>
@@ -6123,7 +6129,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F47C3BC4-135E-49A0-8886-8357248B46C2}">
   <dimension ref="A1:J42"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.875" customWidth="1"/>
     <col min="2" max="2" width="11.625" customWidth="1"/>
@@ -6137,7 +6143,7 @@
     <col min="10" max="10" width="68.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="24" customFormat="1" ht="14.25" customHeight="1">
+    <row r="1" spans="1:10" s="24" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>938</v>
       </c>
@@ -6169,7 +6175,7 @@
         <v>1089</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="14.25" customHeight="1">
+    <row r="2" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>948</v>
       </c>
@@ -6198,7 +6204,7 @@
         <v>1091</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="14.25" customHeight="1">
+    <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>955</v>
       </c>
@@ -6224,7 +6230,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="14.25" customHeight="1">
+    <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>955</v>
       </c>
@@ -6247,7 +6253,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="14.25" customHeight="1">
+    <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>948</v>
       </c>
@@ -6270,7 +6276,7 @@
         <v>954</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="14.25" customHeight="1">
+    <row r="7" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>955</v>
       </c>
@@ -6296,7 +6302,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="14.25" customHeight="1">
+    <row r="8" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>955</v>
       </c>
@@ -6319,7 +6325,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="14.25" customHeight="1">
+    <row r="10" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>955</v>
       </c>
@@ -6345,7 +6351,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="14.25" customHeight="1">
+    <row r="12" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>955</v>
       </c>
@@ -6374,7 +6380,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="14.25" customHeight="1">
+    <row r="13" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>955</v>
       </c>
@@ -6400,7 +6406,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="14.25" customHeight="1">
+    <row r="15" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>948</v>
       </c>
@@ -6426,7 +6432,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="14.25" customHeight="1">
+    <row r="16" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D16" t="s">
         <v>1001</v>
       </c>
@@ -6440,7 +6446,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="14.25" customHeight="1">
+    <row r="18" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>948</v>
       </c>
@@ -6466,7 +6472,7 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="14.25" customHeight="1">
+    <row r="19" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D19" t="s">
         <v>1012</v>
       </c>
@@ -6477,7 +6483,7 @@
         <v>1014</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="14.25" customHeight="1">
+    <row r="21" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>1016</v>
       </c>
@@ -6500,7 +6506,7 @@
         <v>1022</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="14.25" customHeight="1">
+    <row r="23" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>948</v>
       </c>
@@ -6523,7 +6529,7 @@
         <v>1100</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14.25" customHeight="1">
+    <row r="24" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
         <v>1029</v>
       </c>
@@ -6537,7 +6543,7 @@
         <v>1098</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="14.25" customHeight="1">
+    <row r="26" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>948</v>
       </c>
@@ -6563,7 +6569,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="27" spans="1:9" ht="14.25" customHeight="1">
+    <row r="27" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="D27" t="s">
         <v>1038</v>
       </c>
@@ -6571,7 +6577,7 @@
         <v>1039</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="14.25" customHeight="1">
+    <row r="29" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>1016</v>
       </c>
@@ -6594,7 +6600,7 @@
         <v>1045</v>
       </c>
     </row>
-    <row r="32" spans="1:9" ht="14.25" customHeight="1">
+    <row r="32" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>948</v>
       </c>
@@ -6602,7 +6608,7 @@
         <v>1046</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="14.25" customHeight="1">
+    <row r="33" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>948</v>
       </c>
@@ -6613,7 +6619,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="14.25" customHeight="1">
+    <row r="34" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>948</v>
       </c>
@@ -6624,7 +6630,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="14.25" customHeight="1">
+    <row r="36" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>1048</v>
       </c>
@@ -6635,7 +6641,7 @@
         <v>1047</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="14.25" customHeight="1">
+    <row r="38" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>955</v>
       </c>
@@ -6649,7 +6655,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="14.25" customHeight="1">
+    <row r="39" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>955</v>
       </c>
@@ -6663,7 +6669,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="14.25" customHeight="1">
+    <row r="40" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>955</v>
       </c>
@@ -6674,7 +6680,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="14.25" customHeight="1">
+    <row r="42" spans="1:8" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>1101</v>
       </c>
@@ -6691,7 +6697,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{52F3FEB2-DD93-4E94-A954-8EDB8BBDC1E0}">
   <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.875" style="12" customWidth="1"/>
     <col min="2" max="2" width="12.5" style="12" customWidth="1"/>
@@ -6705,7 +6711,7 @@
     <col min="11" max="16384" width="9" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="13" customFormat="1">
+    <row r="1" spans="1:10" s="13" customFormat="1" ht="15" x14ac:dyDescent="0.2">
       <c r="A1" s="13" t="s">
         <v>938</v>
       </c>
@@ -6734,7 +6740,7 @@
         <v>944</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="26.45">
+    <row r="2" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A2" s="10" t="s">
         <v>948</v>
       </c>
@@ -6759,7 +6765,7 @@
       </c>
       <c r="I2" s="10"/>
     </row>
-    <row r="3" spans="1:10" s="31" customFormat="1" ht="15" customHeight="1">
+    <row r="3" spans="1:10" s="31" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="30" t="s">
         <v>955</v>
       </c>
@@ -6769,7 +6775,7 @@
       <c r="C3" s="30" t="s">
         <v>957</v>
       </c>
-      <c r="D3" s="70" t="s">
+      <c r="D3" s="67" t="s">
         <v>958</v>
       </c>
       <c r="E3" s="30"/>
@@ -6789,7 +6795,7 @@
         <v>962</v>
       </c>
     </row>
-    <row r="4" spans="1:10" s="31" customFormat="1" ht="15" customHeight="1">
+    <row r="4" spans="1:10" s="31" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="30" t="s">
         <v>955</v>
       </c>
@@ -6799,7 +6805,7 @@
       <c r="C4" s="30" t="s">
         <v>964</v>
       </c>
-      <c r="D4" s="70"/>
+      <c r="D4" s="67"/>
       <c r="E4" s="30"/>
       <c r="F4" s="30" t="s">
         <v>965</v>
@@ -6817,7 +6823,7 @@
         <v>966</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15" customHeight="1">
+    <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10"/>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
@@ -6831,7 +6837,7 @@
         <v>967</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="27" customHeight="1">
+    <row r="6" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="10" t="s">
         <v>948</v>
       </c>
@@ -6856,7 +6862,7 @@
       </c>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="1:10" ht="15" customHeight="1">
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="10" t="s">
         <v>955</v>
       </c>
@@ -6867,7 +6873,7 @@
         <v>973</v>
       </c>
       <c r="D7" s="34"/>
-      <c r="E7" s="71" t="s">
+      <c r="E7" s="68" t="s">
         <v>364</v>
       </c>
       <c r="F7" s="10" t="s">
@@ -6883,7 +6889,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15" customHeight="1">
+    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="10" t="s">
         <v>955</v>
       </c>
@@ -6894,7 +6900,7 @@
         <v>977</v>
       </c>
       <c r="D8" s="34"/>
-      <c r="E8" s="71"/>
+      <c r="E8" s="68"/>
       <c r="F8" s="10" t="s">
         <v>978</v>
       </c>
@@ -6908,7 +6914,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15" customHeight="1">
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -6919,7 +6925,7 @@
       <c r="H9" s="10"/>
       <c r="I9" s="10"/>
     </row>
-    <row r="10" spans="1:10" ht="15" customHeight="1">
+    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="14" t="s">
         <v>955</v>
       </c>
@@ -6947,7 +6953,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="15" customHeight="1">
+    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="14"/>
       <c r="B11" s="14"/>
       <c r="C11" s="14"/>
@@ -6958,7 +6964,7 @@
       <c r="H11" s="14"/>
       <c r="I11" s="14"/>
     </row>
-    <row r="12" spans="1:10" ht="15" customHeight="1">
+    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="14" t="s">
         <v>955</v>
       </c>
@@ -6986,7 +6992,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="15" customHeight="1">
+    <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
         <v>955</v>
       </c>
@@ -7014,7 +7020,7 @@
         <v>993</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="15" customHeight="1">
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14"/>
       <c r="B14" s="14"/>
       <c r="C14" s="14"/>
@@ -7025,14 +7031,14 @@
       <c r="H14" s="14"/>
       <c r="I14" s="14"/>
     </row>
-    <row r="15" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1">
-      <c r="A15" s="67" t="s">
+    <row r="15" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="69" t="s">
         <v>948</v>
       </c>
-      <c r="B15" s="67" t="s">
+      <c r="B15" s="69" t="s">
         <v>994</v>
       </c>
-      <c r="C15" s="72" t="s">
+      <c r="C15" s="70" t="s">
         <v>995</v>
       </c>
       <c r="D15" s="26" t="s">
@@ -7053,10 +7059,10 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="16" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1">
-      <c r="A16" s="67"/>
-      <c r="B16" s="67"/>
-      <c r="C16" s="67"/>
+    <row r="16" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="69"/>
+      <c r="B16" s="69"/>
+      <c r="C16" s="69"/>
       <c r="D16" s="26" t="s">
         <v>1001</v>
       </c>
@@ -7072,7 +7078,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="14"/>
       <c r="B17" s="14"/>
       <c r="C17" s="14"/>
@@ -7082,14 +7088,14 @@
       <c r="G17" s="14"/>
       <c r="H17" s="17"/>
     </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1">
-      <c r="A18" s="68" t="s">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="65" t="s">
         <v>948</v>
       </c>
-      <c r="B18" s="68" t="s">
+      <c r="B18" s="65" t="s">
         <v>1005</v>
       </c>
-      <c r="C18" s="69" t="s">
+      <c r="C18" s="66" t="s">
         <v>1006</v>
       </c>
       <c r="D18" s="22" t="s">
@@ -7110,10 +7116,10 @@
         <v>1011</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1">
-      <c r="A19" s="68"/>
-      <c r="B19" s="68"/>
-      <c r="C19" s="68"/>
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="65"/>
+      <c r="B19" s="65"/>
+      <c r="C19" s="65"/>
       <c r="D19" s="23" t="s">
         <v>1012</v>
       </c>
@@ -7129,7 +7135,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
       <c r="C20" s="14"/>
@@ -7139,7 +7145,7 @@
       <c r="G20" s="14"/>
       <c r="H20" s="17"/>
     </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1">
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
         <v>1016</v>
       </c>
@@ -7166,7 +7172,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1">
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14"/>
       <c r="B22" s="14"/>
       <c r="C22" s="14"/>
@@ -7177,14 +7183,14 @@
       <c r="H22" s="14"/>
       <c r="I22" s="14"/>
     </row>
-    <row r="23" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1">
-      <c r="A23" s="67" t="s">
+    <row r="23" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="69" t="s">
         <v>948</v>
       </c>
-      <c r="B23" s="67" t="s">
+      <c r="B23" s="69" t="s">
         <v>1024</v>
       </c>
-      <c r="C23" s="67" t="s">
+      <c r="C23" s="69" t="s">
         <v>153</v>
       </c>
       <c r="D23" s="29" t="s">
@@ -7202,10 +7208,10 @@
         <v>1028</v>
       </c>
     </row>
-    <row r="24" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1">
-      <c r="A24" s="67"/>
-      <c r="B24" s="67"/>
-      <c r="C24" s="67"/>
+    <row r="24" spans="1:10" s="27" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="69"/>
+      <c r="B24" s="69"/>
+      <c r="C24" s="69"/>
       <c r="D24" s="26" t="s">
         <v>1029</v>
       </c>
@@ -7221,7 +7227,7 @@
         <v>1004</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1">
+    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="14"/>
       <c r="B25" s="14"/>
       <c r="C25" s="14"/>
@@ -7231,14 +7237,14 @@
       <c r="G25" s="14"/>
       <c r="H25" s="16"/>
     </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1">
-      <c r="A26" s="68" t="s">
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="65" t="s">
         <v>948</v>
       </c>
-      <c r="B26" s="68" t="s">
+      <c r="B26" s="65" t="s">
         <v>1031</v>
       </c>
-      <c r="C26" s="68" t="s">
+      <c r="C26" s="65" t="s">
         <v>1032</v>
       </c>
       <c r="D26" s="16" t="s">
@@ -7257,14 +7263,14 @@
       <c r="I26" s="15" t="s">
         <v>1010</v>
       </c>
-      <c r="J26" s="65" t="s">
+      <c r="J26" s="71" t="s">
         <v>1037</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1">
-      <c r="A27" s="68"/>
-      <c r="B27" s="68"/>
-      <c r="C27" s="68"/>
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="65"/>
+      <c r="B27" s="65"/>
+      <c r="C27" s="65"/>
       <c r="D27" s="18" t="s">
         <v>1038</v>
       </c>
@@ -7277,9 +7283,9 @@
       <c r="I27" s="15" t="s">
         <v>1015</v>
       </c>
-      <c r="J27" s="66"/>
-    </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1">
+      <c r="J27" s="72"/>
+    </row>
+    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="14"/>
       <c r="B28" s="14"/>
       <c r="C28" s="14"/>
@@ -7289,7 +7295,7 @@
       <c r="G28" s="14"/>
       <c r="H28" s="16"/>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="14" t="s">
         <v>1016</v>
       </c>
@@ -7316,7 +7322,7 @@
         <v>1023</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="10"/>
       <c r="B30" s="10"/>
       <c r="C30" s="10"/>
@@ -7327,7 +7333,7 @@
       <c r="H30" s="10"/>
       <c r="I30" s="10"/>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="10"/>
       <c r="B31" s="10"/>
       <c r="C31" s="10"/>
@@ -7338,7 +7344,7 @@
       <c r="H31" s="10"/>
       <c r="I31" s="10"/>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
         <v>948</v>
       </c>
@@ -7353,7 +7359,7 @@
       <c r="H32" s="10"/>
       <c r="I32" s="10"/>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="10" t="s">
         <v>948</v>
       </c>
@@ -7370,7 +7376,7 @@
       </c>
       <c r="I33" s="10"/>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
         <v>948</v>
       </c>
@@ -7387,7 +7393,7 @@
       </c>
       <c r="I34" s="10"/>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -7398,7 +7404,7 @@
       <c r="H35" s="10"/>
       <c r="I35" s="10"/>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="10" t="s">
         <v>1048</v>
       </c>
@@ -7415,7 +7421,7 @@
       </c>
       <c r="I36" s="10"/>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="10"/>
       <c r="B37" s="10"/>
       <c r="C37" s="10"/>
@@ -7426,7 +7432,7 @@
       <c r="H37" s="10"/>
       <c r="I37" s="10"/>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
         <v>955</v>
       </c>
@@ -7445,7 +7451,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="10" t="s">
         <v>955</v>
       </c>
@@ -7464,7 +7470,7 @@
         <v>961</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="10" t="s">
         <v>955</v>
       </c>
@@ -7483,6 +7489,13 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="J26:J27"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
     <mergeCell ref="A18:A19"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="C18:C19"/>
@@ -7491,13 +7504,6 @@
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="C15:C16"/>
-    <mergeCell ref="J26:J27"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7506,7 +7512,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{775FCF44-3854-4073-ABBB-38810E2FE0FC}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
     <col min="2" max="2" width="14.75" customWidth="1"/>
@@ -7516,7 +7522,7 @@
     <col min="6" max="6" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="36" t="s">
         <v>33</v>
       </c>
@@ -7536,7 +7542,7 @@
         <v>1105</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1050</v>
       </c>
@@ -7553,7 +7559,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1050</v>
       </c>
@@ -7573,7 +7579,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1050</v>
       </c>
@@ -7593,7 +7599,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>1050</v>
       </c>
@@ -7613,7 +7619,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>1050</v>
       </c>
@@ -7633,7 +7639,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>1050</v>
       </c>
@@ -7653,7 +7659,7 @@
         <v>1053</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>1050</v>
       </c>
@@ -7684,7 +7690,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC5D690F-892C-4875-BCDC-76BA0A6ABE6A}">
   <dimension ref="A1:AA116"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.125" customWidth="1"/>
     <col min="2" max="2" width="16" style="36" bestFit="1" customWidth="1"/>
@@ -7705,7 +7711,7 @@
     <col min="28" max="28" width="21.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="24" customFormat="1">
+    <row r="1" spans="1:27" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>32</v>
       </c>
@@ -7788,7 +7794,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:27">
+    <row r="2" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>59</v>
       </c>
@@ -7859,7 +7865,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:27">
+    <row r="3" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>74</v>
       </c>
@@ -7915,7 +7921,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:27">
+    <row r="4" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>82</v>
       </c>
@@ -7971,7 +7977,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="5" spans="1:27">
+    <row r="5" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>90</v>
       </c>
@@ -8030,7 +8036,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="7" spans="1:27">
+    <row r="6" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="7" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>98</v>
       </c>
@@ -8104,7 +8111,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="8" spans="1:27">
+    <row r="8" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>107</v>
       </c>
@@ -8160,7 +8167,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:27">
+    <row r="9" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>112</v>
       </c>
@@ -8216,7 +8223,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="10" spans="1:27">
+    <row r="10" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>117</v>
       </c>
@@ -8275,7 +8282,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="12" spans="1:27">
+    <row r="11" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>122</v>
       </c>
@@ -8325,7 +8333,8 @@
         <v>123</v>
       </c>
     </row>
-    <row r="14" spans="1:27">
+    <row r="13" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="14" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>126</v>
       </c>
@@ -8366,7 +8375,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="15" spans="1:27">
+    <row r="15" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>131</v>
       </c>
@@ -8401,7 +8410,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:27">
+    <row r="16" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>134</v>
       </c>
@@ -8436,7 +8445,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:27">
+    <row r="17" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>137</v>
       </c>
@@ -8471,7 +8480,8 @@
         <v>138</v>
       </c>
     </row>
-    <row r="19" spans="1:27">
+    <row r="18" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="19" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>140</v>
       </c>
@@ -8518,7 +8528,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:27">
+    <row r="20" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>144</v>
       </c>
@@ -8553,7 +8563,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="21" spans="1:27">
+    <row r="21" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>146</v>
       </c>
@@ -8588,7 +8598,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="22" spans="1:27">
+    <row r="22" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>148</v>
       </c>
@@ -8623,7 +8633,8 @@
         <v>150</v>
       </c>
     </row>
-    <row r="24" spans="1:27">
+    <row r="23" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>151</v>
       </c>
@@ -8679,7 +8690,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="25" spans="1:27">
+    <row r="25" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>156</v>
       </c>
@@ -8732,7 +8743,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="26" spans="1:27" ht="13.5" customHeight="1">
+    <row r="26" spans="1:27" ht="13.5" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>159</v>
       </c>
@@ -8791,7 +8802,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="27" spans="1:27">
+    <row r="27" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>166</v>
       </c>
@@ -8847,7 +8858,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="28" spans="1:27">
+    <row r="28" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>171</v>
       </c>
@@ -8900,7 +8911,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="29" spans="1:27">
+    <row r="29" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>177</v>
       </c>
@@ -8938,7 +8949,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:27">
+    <row r="30" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>180</v>
       </c>
@@ -8985,7 +8996,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="31" spans="1:27">
+    <row r="31" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>185</v>
       </c>
@@ -9029,7 +9040,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="32" spans="1:27">
+    <row r="32" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>189</v>
       </c>
@@ -9076,7 +9087,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="33" spans="1:27">
+    <row r="33" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>193</v>
       </c>
@@ -9126,7 +9137,8 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" spans="1:27">
+    <row r="34" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="35" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>196</v>
       </c>
@@ -9173,7 +9185,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="36" spans="1:27">
+    <row r="36" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>203</v>
       </c>
@@ -9205,7 +9217,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="37" spans="1:27">
+    <row r="37" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>206</v>
       </c>
@@ -9234,7 +9246,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="38" spans="1:27">
+    <row r="38" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>209</v>
       </c>
@@ -9263,7 +9275,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" spans="1:27">
+    <row r="39" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="40" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>210</v>
       </c>
@@ -9310,7 +9323,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="41" spans="1:27">
+    <row r="41" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>216</v>
       </c>
@@ -9339,7 +9352,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="42" spans="1:27">
+    <row r="42" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>219</v>
       </c>
@@ -9368,7 +9381,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="43" spans="1:27">
+    <row r="43" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>221</v>
       </c>
@@ -9397,7 +9410,8 @@
         <v>223</v>
       </c>
     </row>
-    <row r="45" spans="1:27">
+    <row r="44" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>224</v>
       </c>
@@ -9444,7 +9458,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="46" spans="1:27">
+    <row r="46" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>229</v>
       </c>
@@ -9488,7 +9502,8 @@
         <v>233</v>
       </c>
     </row>
-    <row r="48" spans="1:27" ht="15" customHeight="1">
+    <row r="47" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:27" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>234</v>
       </c>
@@ -9538,7 +9553,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="49" spans="1:27">
+    <row r="49" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>239</v>
       </c>
@@ -9585,7 +9600,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="50" spans="1:27">
+    <row r="50" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>244</v>
       </c>
@@ -9632,7 +9647,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="51" spans="1:27">
+    <row r="51" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>246</v>
       </c>
@@ -9679,7 +9694,8 @@
         <v>243</v>
       </c>
     </row>
-    <row r="53" spans="1:27">
+    <row r="52" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="53" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>248</v>
       </c>
@@ -9729,7 +9745,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="54" spans="1:27">
+    <row r="54" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>253</v>
       </c>
@@ -9776,7 +9792,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="55" spans="1:27">
+    <row r="55" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>257</v>
       </c>
@@ -9832,7 +9848,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="56" spans="1:27">
+    <row r="56" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>261</v>
       </c>
@@ -9885,7 +9901,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="57" spans="1:27">
+    <row r="57" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>265</v>
       </c>
@@ -9938,7 +9954,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="58" spans="1:27">
+    <row r="58" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>269</v>
       </c>
@@ -9994,7 +10010,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="59" spans="1:27">
+    <row r="59" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>273</v>
       </c>
@@ -10044,7 +10060,8 @@
         <v>277</v>
       </c>
     </row>
-    <row r="61" spans="1:27">
+    <row r="60" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="61" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>278</v>
       </c>
@@ -10067,7 +10084,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:27">
+    <row r="62" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>281</v>
       </c>
@@ -10090,7 +10107,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="63" spans="1:27">
+    <row r="63" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>283</v>
       </c>
@@ -10113,7 +10130,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="64" spans="1:27">
+    <row r="64" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>285</v>
       </c>
@@ -10136,7 +10153,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="66" spans="1:27">
+    <row r="65" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="66" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>286</v>
       </c>
@@ -10159,7 +10177,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:27">
+    <row r="67" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>288</v>
       </c>
@@ -10182,7 +10200,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="1:27">
+    <row r="68" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>290</v>
       </c>
@@ -10205,7 +10223,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="69" spans="1:27">
+    <row r="69" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>292</v>
       </c>
@@ -10228,7 +10246,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="71" spans="1:27">
+    <row r="70" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="71" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>293</v>
       </c>
@@ -10260,7 +10279,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="72" spans="1:27">
+    <row r="72" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>296</v>
       </c>
@@ -10283,7 +10302,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:27">
+    <row r="73" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>298</v>
       </c>
@@ -10303,7 +10322,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="74" spans="1:27">
+    <row r="74" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>299</v>
       </c>
@@ -10323,7 +10342,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="76" spans="1:27">
+    <row r="75" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="76" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>300</v>
       </c>
@@ -10367,7 +10387,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="77" spans="1:27">
+    <row r="77" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>306</v>
       </c>
@@ -10384,7 +10404,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="1:27">
+    <row r="78" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>307</v>
       </c>
@@ -10401,7 +10421,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="79" spans="1:27">
+    <row r="79" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>308</v>
       </c>
@@ -10418,7 +10438,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="81" spans="1:27">
+    <row r="80" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="81" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>309</v>
       </c>
@@ -10465,7 +10486,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="82" spans="1:27">
+    <row r="82" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>315</v>
       </c>
@@ -10509,7 +10530,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="83" spans="1:27">
+    <row r="83" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>319</v>
       </c>
@@ -10556,7 +10577,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="84" spans="1:27">
+    <row r="84" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>324</v>
       </c>
@@ -10600,7 +10621,8 @@
         <v>327</v>
       </c>
     </row>
-    <row r="86" spans="1:27">
+    <row r="85" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="86" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>328</v>
       </c>
@@ -10647,7 +10669,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="87" spans="1:27">
+    <row r="87" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>332</v>
       </c>
@@ -10691,7 +10713,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="88" spans="1:27">
+    <row r="88" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>335</v>
       </c>
@@ -10735,7 +10757,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="89" spans="1:27">
+    <row r="89" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>339</v>
       </c>
@@ -10776,7 +10798,9 @@
         <v>340</v>
       </c>
     </row>
-    <row r="92" spans="1:27">
+    <row r="90" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="91" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="92" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>342</v>
       </c>
@@ -10829,7 +10853,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="93" spans="1:27">
+    <row r="93" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>349</v>
       </c>
@@ -10855,7 +10879,8 @@
         <v>351</v>
       </c>
     </row>
-    <row r="95" spans="1:27">
+    <row r="94" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="95" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>352</v>
       </c>
@@ -10902,7 +10927,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="96" spans="1:27">
+    <row r="96" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>356</v>
       </c>
@@ -10922,7 +10947,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="97" spans="1:27">
+    <row r="97" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>358</v>
       </c>
@@ -10942,7 +10967,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="98" spans="1:27">
+    <row r="98" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>360</v>
       </c>
@@ -10962,7 +10987,8 @@
         <v>93</v>
       </c>
     </row>
-    <row r="100" spans="1:27">
+    <row r="99" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
+    <row r="100" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>362</v>
       </c>
@@ -11009,7 +11035,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="101" spans="1:27">
+    <row r="101" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>366</v>
       </c>
@@ -11029,7 +11055,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="102" spans="1:27">
+    <row r="102" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>368</v>
       </c>
@@ -11049,7 +11075,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="103" spans="1:27">
+    <row r="103" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>370</v>
       </c>
@@ -11069,7 +11095,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="105" spans="1:27">
+    <row r="105" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>372</v>
       </c>
@@ -11101,7 +11127,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="106" spans="1:27">
+    <row r="106" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>378</v>
       </c>
@@ -11130,12 +11156,12 @@
         <v>377</v>
       </c>
     </row>
-    <row r="107" spans="1:27">
+    <row r="107" spans="1:27" x14ac:dyDescent="0.2">
       <c r="AA107" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="108" spans="1:27">
+    <row r="108" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>380</v>
       </c>
@@ -11167,7 +11193,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="109" spans="1:27">
+    <row r="109" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>384</v>
       </c>
@@ -11196,12 +11222,12 @@
         <v>377</v>
       </c>
     </row>
-    <row r="110" spans="1:27">
+    <row r="110" spans="1:27" x14ac:dyDescent="0.2">
       <c r="AA110" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="111" spans="1:27">
+    <row r="111" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>386</v>
       </c>
@@ -11233,7 +11259,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="112" spans="1:27">
+    <row r="112" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>390</v>
       </c>
@@ -11262,7 +11288,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="114" spans="1:15">
+    <row r="114" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>392</v>
       </c>
@@ -11288,7 +11314,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="115" spans="1:15">
+    <row r="115" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>394</v>
       </c>
@@ -11314,7 +11340,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="116" spans="1:15">
+    <row r="116" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>395</v>
       </c>
@@ -11355,7 +11381,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F9CED11-E3D2-4EC3-A4A4-2AC4728D182C}">
   <dimension ref="A1:P11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.25" customWidth="1"/>
     <col min="2" max="2" width="15.875" customWidth="1"/>
@@ -11375,7 +11401,7 @@
     <col min="16" max="16" width="10.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="24" customFormat="1">
+    <row r="1" spans="1:16" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>396</v>
       </c>
@@ -11425,7 +11451,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>400</v>
       </c>
@@ -11472,7 +11498,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>411</v>
       </c>
@@ -11498,7 +11524,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>416</v>
       </c>
@@ -11524,7 +11550,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>421</v>
       </c>
@@ -11550,7 +11576,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>426</v>
       </c>
@@ -11576,7 +11602,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>431</v>
       </c>
@@ -11602,7 +11628,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>436</v>
       </c>
@@ -11637,7 +11663,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>440</v>
       </c>
@@ -11660,7 +11686,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>443</v>
       </c>
@@ -11692,7 +11718,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>446</v>
       </c>
@@ -11728,7 +11754,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:Q63"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="9.375" bestFit="1" customWidth="1"/>
@@ -11749,7 +11775,7 @@
     <col min="17" max="17" width="22.875" style="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="24" customFormat="1">
+    <row r="1" spans="1:17" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>32</v>
       </c>
@@ -11802,7 +11828,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:17">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>452</v>
       </c>
@@ -11840,7 +11866,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="3" spans="1:17">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>459</v>
       </c>
@@ -11860,7 +11886,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:17">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>461</v>
       </c>
@@ -11880,7 +11906,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:17">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>463</v>
       </c>
@@ -11900,7 +11926,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:17">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>465</v>
       </c>
@@ -11920,7 +11946,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="7" spans="1:17">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>469</v>
       </c>
@@ -11940,7 +11966,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>473</v>
       </c>
@@ -11963,7 +11989,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="9" spans="1:17">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>476</v>
       </c>
@@ -11986,7 +12012,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="11" spans="1:17">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>479</v>
       </c>
@@ -12030,7 +12056,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="12" spans="1:17">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>486</v>
       </c>
@@ -12050,7 +12076,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:17">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>487</v>
       </c>
@@ -12070,7 +12096,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:17">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>488</v>
       </c>
@@ -12090,7 +12116,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:17">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>489</v>
       </c>
@@ -12110,7 +12136,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="16" spans="1:17">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>490</v>
       </c>
@@ -12130,7 +12156,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="17" spans="1:17">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>491</v>
       </c>
@@ -12153,7 +12179,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="18" spans="1:17">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>492</v>
       </c>
@@ -12176,7 +12202,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="20" spans="1:17">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>493</v>
       </c>
@@ -12214,7 +12240,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="21" spans="1:17">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>499</v>
       </c>
@@ -12234,7 +12260,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>501</v>
       </c>
@@ -12254,7 +12280,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="23" spans="1:17">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>503</v>
       </c>
@@ -12274,7 +12300,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="24" spans="1:17">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>505</v>
       </c>
@@ -12294,7 +12320,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="25" spans="1:17">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>507</v>
       </c>
@@ -12314,7 +12340,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="26" spans="1:17">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>509</v>
       </c>
@@ -12334,7 +12360,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="27" spans="1:17">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>511</v>
       </c>
@@ -12354,7 +12380,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="29" spans="1:17">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>512</v>
       </c>
@@ -12398,7 +12424,7 @@
         <v>518</v>
       </c>
     </row>
-    <row r="30" spans="1:17" ht="15" customHeight="1">
+    <row r="30" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>519</v>
       </c>
@@ -12427,7 +12453,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="31" spans="1:17">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>523</v>
       </c>
@@ -12447,7 +12473,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="32" spans="1:17">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>524</v>
       </c>
@@ -12467,7 +12493,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="33" spans="1:17">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>525</v>
       </c>
@@ -12487,7 +12513,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="34" spans="1:17">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>526</v>
       </c>
@@ -12507,7 +12533,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="35" spans="1:17">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>528</v>
       </c>
@@ -12524,7 +12550,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:17">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>529</v>
       </c>
@@ -12541,7 +12567,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="38" spans="1:17">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>530</v>
       </c>
@@ -12582,7 +12608,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="39" spans="1:17">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>536</v>
       </c>
@@ -12602,7 +12628,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:17">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>537</v>
       </c>
@@ -12622,7 +12648,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:17">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>538</v>
       </c>
@@ -12642,7 +12668,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="42" spans="1:17">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>539</v>
       </c>
@@ -12662,7 +12688,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="43" spans="1:17">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>540</v>
       </c>
@@ -12682,7 +12708,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="44" spans="1:17">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>541</v>
       </c>
@@ -12702,7 +12728,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="45" spans="1:17">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>542</v>
       </c>
@@ -12722,7 +12748,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="47" spans="1:17">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>543</v>
       </c>
@@ -12760,7 +12786,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="48" spans="1:17">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>548</v>
       </c>
@@ -12780,7 +12806,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="49" spans="1:17">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>549</v>
       </c>
@@ -12800,7 +12826,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="50" spans="1:17">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>550</v>
       </c>
@@ -12820,7 +12846,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="51" spans="1:17">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>551</v>
       </c>
@@ -12840,7 +12866,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="52" spans="1:17">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>552</v>
       </c>
@@ -12860,7 +12886,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="53" spans="1:17">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>553</v>
       </c>
@@ -12880,7 +12906,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="54" spans="1:17">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>554</v>
       </c>
@@ -12900,7 +12926,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="56" spans="1:17">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>555</v>
       </c>
@@ -12938,7 +12964,7 @@
         <v>560</v>
       </c>
     </row>
-    <row r="57" spans="1:17">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>561</v>
       </c>
@@ -12961,7 +12987,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="58" spans="1:17">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>563</v>
       </c>
@@ -12981,7 +13007,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="59" spans="1:17">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>564</v>
       </c>
@@ -13001,7 +13027,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="60" spans="1:17">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>565</v>
       </c>
@@ -13021,7 +13047,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="61" spans="1:17">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>566</v>
       </c>
@@ -13041,7 +13067,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="62" spans="1:17">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>567</v>
       </c>
@@ -13064,7 +13090,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="63" spans="1:17">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>568</v>
       </c>
@@ -13101,7 +13127,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1FB411F-E198-4F5E-B603-AEE89BDA3DC7}">
   <dimension ref="A1:D65"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17.75" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.875" customWidth="1"/>
@@ -13110,7 +13136,7 @@
     <col min="5" max="5" width="22.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.6">
+    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="39" t="s">
         <v>569</v>
       </c>
@@ -13121,7 +13147,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="24">
         <v>1</v>
       </c>
@@ -13132,7 +13158,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="24">
         <v>2</v>
       </c>
@@ -13143,7 +13169,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="24">
         <v>3</v>
       </c>
@@ -13154,7 +13180,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="24">
         <v>4</v>
       </c>
@@ -13165,7 +13191,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="24">
         <v>5</v>
       </c>
@@ -13176,7 +13202,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="24">
         <v>6</v>
       </c>
@@ -13187,7 +13213,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="24">
         <v>7</v>
       </c>
@@ -13198,7 +13224,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="24">
         <v>8</v>
       </c>
@@ -13209,7 +13235,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="24">
         <v>9</v>
       </c>
@@ -13220,7 +13246,7 @@
         <v>589</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="24">
         <v>10</v>
       </c>
@@ -13231,7 +13257,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="24">
         <v>11</v>
       </c>
@@ -13242,7 +13268,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="24">
         <v>12</v>
       </c>
@@ -13253,7 +13279,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="24">
         <v>13</v>
       </c>
@@ -13264,7 +13290,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="24">
         <v>14</v>
       </c>
@@ -13275,7 +13301,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="24">
         <v>15</v>
       </c>
@@ -13286,247 +13312,247 @@
         <v>601</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="24">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="24">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A19" s="24">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="24">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="24">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="24">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="24">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="24">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="24">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="24">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="24">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="24">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A29" s="24">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A30" s="24">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="24">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A32" s="24">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A33" s="24">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A34" s="24">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A35" s="24">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A36" s="24">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A37" s="24">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A38" s="24">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A39" s="24">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A40" s="24">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A41" s="24">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A42" s="24">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A43" s="24">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A44" s="24">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A45" s="24">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A46" s="24">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A47" s="24">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A48" s="24">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="24">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="24">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="24">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="24">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="24">
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="24">
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="24">
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:1">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="24">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:1">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" s="24">
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:1">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A58" s="24">
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:1">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A59" s="24">
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:1">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A60" s="24">
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" s="24">
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="24">
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A63" s="24">
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A64" s="24">
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:1">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A65" s="24">
         <v>64</v>
       </c>
@@ -13539,7 +13565,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BBF9283-EF03-4203-B1F1-7C2AF5F0A14C}">
   <dimension ref="A1:W35"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.75" customWidth="1"/>
@@ -13566,7 +13592,7 @@
     <col min="23" max="23" width="10.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" s="24" customFormat="1">
+    <row r="1" spans="1:23" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>32</v>
       </c>
@@ -13637,7 +13663,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>606</v>
       </c>
@@ -13663,7 +13689,7 @@
         <v>609</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>610</v>
       </c>
@@ -13689,7 +13715,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>614</v>
       </c>
@@ -13715,7 +13741,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>618</v>
       </c>
@@ -13741,7 +13767,7 @@
         <v>621</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>622</v>
       </c>
@@ -13767,7 +13793,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>626</v>
       </c>
@@ -13793,7 +13819,7 @@
         <v>629</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>630</v>
       </c>
@@ -13819,7 +13845,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="10" spans="1:23">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>634</v>
       </c>
@@ -13845,7 +13871,7 @@
         <v>637</v>
       </c>
     </row>
-    <row r="12" spans="1:23">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>638</v>
       </c>
@@ -13871,7 +13897,7 @@
         <v>640</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>641</v>
       </c>
@@ -13897,7 +13923,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>644</v>
       </c>
@@ -13923,7 +13949,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>647</v>
       </c>
@@ -13949,7 +13975,7 @@
         <v>649</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>650</v>
       </c>
@@ -13975,7 +14001,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="17" spans="1:12">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>653</v>
       </c>
@@ -14001,7 +14027,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="19" spans="1:12">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>656</v>
       </c>
@@ -14027,7 +14053,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="20" spans="1:12">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>660</v>
       </c>
@@ -14053,7 +14079,7 @@
         <v>663</v>
       </c>
     </row>
-    <row r="22" spans="1:12">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>664</v>
       </c>
@@ -14085,7 +14111,7 @@
         <v>668</v>
       </c>
     </row>
-    <row r="23" spans="1:12">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>669</v>
       </c>
@@ -14117,7 +14143,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="25" spans="1:12">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>674</v>
       </c>
@@ -14146,7 +14172,7 @@
         <v>679</v>
       </c>
     </row>
-    <row r="26" spans="1:12">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>680</v>
       </c>
@@ -14175,7 +14201,7 @@
         <v>684</v>
       </c>
     </row>
-    <row r="28" spans="1:12">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>685</v>
       </c>
@@ -14204,12 +14230,12 @@
         <v>689</v>
       </c>
     </row>
-    <row r="29" spans="1:12">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B29">
         <v>107</v>
       </c>
     </row>
-    <row r="31" spans="1:12">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>690</v>
       </c>
@@ -14229,7 +14255,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="32" spans="1:12">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>694</v>
       </c>
@@ -14249,7 +14275,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>696</v>
       </c>
@@ -14269,7 +14295,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>698</v>
       </c>
@@ -14302,7 +14328,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{555AD50E-91E1-4D37-9A39-B0F1C8CD7595}">
   <dimension ref="A1:U45"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12.5" customWidth="1"/>
     <col min="2" max="2" width="8.75" customWidth="1"/>
@@ -14327,7 +14353,7 @@
     <col min="21" max="21" width="34.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" s="24" customFormat="1">
+    <row r="1" spans="1:21" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>700</v>
       </c>
@@ -14392,7 +14418,7 @@
         <v>708</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>709</v>
       </c>
@@ -14424,7 +14450,7 @@
         <v>714</v>
       </c>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>715</v>
       </c>
@@ -14447,7 +14473,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>717</v>
       </c>
@@ -14482,7 +14508,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>720</v>
       </c>
@@ -14505,7 +14531,7 @@
         <v>719</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>721</v>
       </c>
@@ -14540,7 +14566,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>727</v>
       </c>
@@ -14569,7 +14595,7 @@
         <v>726</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>730</v>
       </c>
@@ -14601,7 +14627,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>732</v>
       </c>
@@ -14627,7 +14653,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>733</v>
       </c>
@@ -14662,7 +14688,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="13" spans="1:21">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>738</v>
       </c>
@@ -14688,7 +14714,7 @@
         <v>737</v>
       </c>
     </row>
-    <row r="14" spans="1:21">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>741</v>
       </c>
@@ -14720,7 +14746,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>742</v>
       </c>
@@ -14743,7 +14769,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>743</v>
       </c>
@@ -14778,7 +14804,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>748</v>
       </c>
@@ -14804,7 +14830,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>750</v>
       </c>
@@ -14836,7 +14862,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>752</v>
       </c>
@@ -14859,7 +14885,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>753</v>
       </c>
@@ -14897,7 +14923,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>758</v>
       </c>
@@ -14920,7 +14946,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>759</v>
       </c>
@@ -14958,7 +14984,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="25" spans="1:21">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>761</v>
       </c>
@@ -14984,7 +15010,7 @@
         <v>760</v>
       </c>
     </row>
-    <row r="27" spans="1:21">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>762</v>
       </c>
@@ -15016,7 +15042,7 @@
         <v>766</v>
       </c>
     </row>
-    <row r="28" spans="1:21">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>767</v>
       </c>
@@ -15039,7 +15065,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="29" spans="1:21">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>768</v>
       </c>
@@ -15068,7 +15094,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="30" spans="1:21">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>769</v>
       </c>
@@ -15088,7 +15114,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="32" spans="1:21">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>770</v>
       </c>
@@ -15123,7 +15149,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="33" spans="1:21">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>774</v>
       </c>
@@ -15146,7 +15172,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="34" spans="1:21">
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>775</v>
       </c>
@@ -15178,7 +15204,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="35" spans="1:21">
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>776</v>
       </c>
@@ -15198,7 +15224,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:21">
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>777</v>
       </c>
@@ -15233,7 +15259,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="38" spans="1:21">
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>785</v>
       </c>
@@ -15256,7 +15282,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="39" spans="1:21">
+    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>786</v>
       </c>
@@ -15285,7 +15311,7 @@
         <v>782</v>
       </c>
     </row>
-    <row r="40" spans="1:21">
+    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>787</v>
       </c>
@@ -15305,7 +15331,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="42" spans="1:21">
+    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>788</v>
       </c>
@@ -15337,7 +15363,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="43" spans="1:21">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>791</v>
       </c>
@@ -15360,7 +15386,7 @@
         <v>780</v>
       </c>
     </row>
-    <row r="44" spans="1:21">
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>792</v>
       </c>
@@ -15389,7 +15415,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="45" spans="1:21">
+    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>793</v>
       </c>
@@ -15425,7 +15451,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M58"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.125" style="24" customWidth="1"/>
     <col min="2" max="2" width="15.25" style="24" bestFit="1" customWidth="1"/>
@@ -15439,7 +15465,7 @@
     <col min="14" max="16384" width="9" style="24"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="32" customFormat="1" ht="14.45">
+    <row r="1" spans="1:13" s="32" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A1" s="32" t="s">
         <v>794</v>
       </c>
@@ -15465,7 +15491,7 @@
         <v>801</v>
       </c>
     </row>
-    <row r="2" spans="1:13">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
         <v>802</v>
       </c>
@@ -15491,7 +15517,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="24" t="s">
         <v>807</v>
       </c>
@@ -15514,7 +15540,7 @@
         <v>809</v>
       </c>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="24" t="s">
         <v>810</v>
       </c>
@@ -15534,7 +15560,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="24" t="s">
         <v>813</v>
       </c>
@@ -15557,7 +15583,7 @@
         <v>816</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="24" t="s">
         <v>817</v>
       </c>
@@ -15577,7 +15603,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="24" t="s">
         <v>821</v>
       </c>
@@ -15585,7 +15611,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="24" t="s">
         <v>779</v>
       </c>
@@ -15608,7 +15634,7 @@
         <v>826</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="24" t="s">
         <v>827</v>
       </c>
@@ -15616,7 +15642,7 @@
         <v>764</v>
       </c>
     </row>
-    <row r="10" spans="1:13">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="24" t="s">
         <v>828</v>
       </c>
@@ -15624,7 +15650,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="11" spans="1:13">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="24" t="s">
         <v>830</v>
       </c>
@@ -15632,7 +15658,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="24" t="s">
         <v>832</v>
       </c>
@@ -15640,7 +15666,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="24" t="s">
         <v>834</v>
       </c>
@@ -15648,7 +15674,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="24" t="s">
         <v>836</v>
       </c>
@@ -15656,7 +15682,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="24" t="s">
         <v>838</v>
       </c>
@@ -15664,7 +15690,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" ht="15" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
         <v>840</v>
       </c>
@@ -15676,7 +15702,7 @@
       </c>
       <c r="J16" s="64"/>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
         <v>843</v>
       </c>
@@ -15690,7 +15716,7 @@
         <v>846</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>847</v>
       </c>
@@ -15704,7 +15730,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>849</v>
       </c>
@@ -15718,7 +15744,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>852</v>
       </c>
@@ -15732,7 +15758,7 @@
         <v>855</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" ht="15" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>856</v>
       </c>
@@ -15746,7 +15772,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="24" t="s">
         <v>858</v>
       </c>
@@ -15754,7 +15780,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="24" t="s">
         <v>859</v>
       </c>
@@ -15762,7 +15788,7 @@
         <v>860</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="24" t="s">
         <v>763</v>
       </c>
@@ -15770,7 +15796,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="24" t="s">
         <v>862</v>
       </c>
@@ -15778,7 +15804,7 @@
         <v>805</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="24" t="s">
         <v>863</v>
       </c>
@@ -15786,7 +15812,7 @@
         <v>864</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="24" t="s">
         <v>865</v>
       </c>
@@ -15794,7 +15820,7 @@
         <v>866</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="24" t="s">
         <v>867</v>
       </c>
@@ -15802,7 +15828,7 @@
         <v>868</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="24" t="s">
         <v>869</v>
       </c>
@@ -15810,7 +15836,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="24" t="s">
         <v>871</v>
       </c>
@@ -15818,7 +15844,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="24" t="s">
         <v>873</v>
       </c>
@@ -15826,7 +15852,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="24" t="s">
         <v>875</v>
       </c>
@@ -15834,7 +15860,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="33" spans="1:13">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="24" t="s">
         <v>876</v>
       </c>
@@ -15842,7 +15868,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="34" spans="1:13">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="24" t="s">
         <v>878</v>
       </c>
@@ -15850,7 +15876,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="35" spans="1:13">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="24" t="s">
         <v>880</v>
       </c>
@@ -15858,7 +15884,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="36" spans="1:13">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="24" t="s">
         <v>882</v>
       </c>
@@ -15866,7 +15892,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="37" spans="1:13">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="24" t="s">
         <v>884</v>
       </c>
@@ -15874,7 +15900,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="38" spans="1:13">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="24" t="s">
         <v>886</v>
       </c>
@@ -15885,7 +15911,7 @@
         <v>887</v>
       </c>
     </row>
-    <row r="39" spans="1:13">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="24" t="s">
         <v>888</v>
       </c>
@@ -15896,7 +15922,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="40" spans="1:13">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="24" t="s">
         <v>891</v>
       </c>
@@ -15907,7 +15933,7 @@
         <v>893</v>
       </c>
     </row>
-    <row r="41" spans="1:13">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="24" t="s">
         <v>894</v>
       </c>
@@ -15918,7 +15944,7 @@
         <v>895</v>
       </c>
     </row>
-    <row r="42" spans="1:13">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="24" t="s">
         <v>896</v>
       </c>
@@ -15929,7 +15955,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="43" spans="1:13">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="24" t="s">
         <v>898</v>
       </c>
@@ -15940,7 +15966,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="44" spans="1:13">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="24" t="s">
         <v>901</v>
       </c>
@@ -15948,7 +15974,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="45" spans="1:13">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="24" t="s">
         <v>903</v>
       </c>
@@ -15956,7 +15982,7 @@
         <v>904</v>
       </c>
     </row>
-    <row r="46" spans="1:13">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="24" t="s">
         <v>905</v>
       </c>
@@ -15964,7 +15990,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="47" spans="1:13">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="24" t="s">
         <v>907</v>
       </c>
@@ -15972,7 +15998,7 @@
         <v>908</v>
       </c>
     </row>
-    <row r="48" spans="1:13">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="24" t="s">
         <v>909</v>
       </c>
@@ -15980,7 +16006,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="49" spans="1:2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" s="24" t="s">
         <v>911</v>
       </c>
@@ -15988,7 +16014,7 @@
         <v>912</v>
       </c>
     </row>
-    <row r="50" spans="1:2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="24" t="s">
         <v>913</v>
       </c>
@@ -15996,7 +16022,7 @@
         <v>914</v>
       </c>
     </row>
-    <row r="51" spans="1:2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" s="24" t="s">
         <v>915</v>
       </c>
@@ -16004,7 +16030,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="52" spans="1:2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" s="24" t="s">
         <v>917</v>
       </c>
@@ -16012,7 +16038,7 @@
         <v>918</v>
       </c>
     </row>
-    <row r="53" spans="1:2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" s="24" t="s">
         <v>919</v>
       </c>
@@ -16020,7 +16046,7 @@
         <v>920</v>
       </c>
     </row>
-    <row r="54" spans="1:2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" s="24" t="s">
         <v>843</v>
       </c>
@@ -16028,7 +16054,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="55" spans="1:2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" s="24" t="s">
         <v>921</v>
       </c>
@@ -16036,7 +16062,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="56" spans="1:2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" s="24" t="s">
         <v>923</v>
       </c>
@@ -16044,7 +16070,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="57" spans="1:2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" s="24" t="s">
         <v>924</v>
       </c>
@@ -16052,7 +16078,7 @@
         <v>925</v>
       </c>
     </row>
-    <row r="58" spans="1:2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" s="24" t="s">
         <v>926</v>
       </c>
@@ -16073,7 +16099,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7B86970-B218-4E9A-ACEA-2014FDEB1916}">
   <dimension ref="A1:Y3"/>
-  <sheetFormatPr defaultRowHeight="13.9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.75" customWidth="1"/>
     <col min="2" max="2" width="13.625" hidden="1" customWidth="1"/>
@@ -16100,7 +16126,7 @@
     <col min="25" max="25" width="32.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="24" customFormat="1">
+    <row r="1" spans="1:25" s="24" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="24" t="s">
         <v>32</v>
       </c>
@@ -16177,7 +16203,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>929</v>
       </c>
@@ -16203,7 +16229,7 @@
         <v>934</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>935</v>
       </c>
@@ -16466,6 +16492,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="757b9e3d-71f1-4cf0-a356-ce1799a3ba84" xsi:nil="true"/>
@@ -16533,23 +16568,46 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{510D5911-AE72-4B88-9FAD-5025643DD754}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{510D5911-AE72-4B88-9FAD-5025643DD754}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b0df0e66-3fca-4c0a-9027-3403a9017d61"/>
+    <ds:schemaRef ds:uri="757b9e3d-71f1-4cf0-a356-ce1799a3ba84"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{163AA8D4-3DDD-4666-A9B4-D1E5B7146C17}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D469EB51-8C6D-4182-9B1F-AA59082D2CCD}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D469EB51-8C6D-4182-9B1F-AA59082D2CCD}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{163AA8D4-3DDD-4666-A9B4-D1E5B7146C17}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="757b9e3d-71f1-4cf0-a356-ce1799a3ba84"/>
+    <ds:schemaRef ds:uri="b0df0e66-3fca-4c0a-9027-3403a9017d61"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{6e4d9da4-fe0d-41ed-9e5c-09814f1447dd}" enabled="1" method="Standard" siteId="{9e5488e2-e838-44f6-886c-c7608242767e}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
Implement CSV import functionality for device creation, allowing devices to be added to an "Unassigned" holding site if no matching city/site is found. Enhance inventory API to protect the holding bin from deletion and renaming. Update UI to support CSV import and display results, including a template for CSV structure. Modify tests to validate the new import process and holding bin protections.
</commit_message>
<xml_diff>
--- a/Example Docs/Newsnation Global Path Naming.xlsx
+++ b/Example Docs/Newsnation Global Path Naming.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/26CA7F966D4A52C6/Code/NexNOC/Example Docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2898" documentId="14_{AA77E42B-1188-4023-99CE-412A287F8599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF44593C-D8D5-49FA-81CF-072765EEB763}"/>
+  <xr:revisionPtr revIDLastSave="2899" documentId="14_{AA77E42B-1188-4023-99CE-412A287F8599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47D315A4-C39B-4FF7-B39B-AAE632E5555D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="15720" tabRatio="816" activeTab="1" xr2:uid="{98E875BD-AF76-45D8-B210-E932B4556ABF}"/>
   </bookViews>
@@ -4336,7 +4336,7 @@
   <autoFilter ref="A1:AA103" xr:uid="{1E6FE14C-CA21-486E-B817-8C185D5E3288}">
     <filterColumn colId="2">
       <filters>
-        <filter val="WDCW"/>
+        <filter val="ATL CW"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -10061,7 +10061,7 @@
       </c>
     </row>
     <row r="60" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="61" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>278</v>
       </c>
@@ -10084,7 +10084,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>281</v>
       </c>
@@ -10107,7 +10107,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="63" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>283</v>
       </c>
@@ -10130,7 +10130,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="64" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>285</v>
       </c>
@@ -10154,7 +10154,7 @@
       </c>
     </row>
     <row r="65" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="66" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>286</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="67" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>288</v>
       </c>
@@ -10200,7 +10200,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="68" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>290</v>
       </c>
@@ -10223,7 +10223,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="69" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>292</v>
       </c>
@@ -10247,7 +10247,7 @@
       </c>
     </row>
     <row r="70" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>293</v>
       </c>
@@ -10279,7 +10279,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="72" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>296</v>
       </c>
@@ -10302,7 +10302,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>298</v>
       </c>
@@ -10322,7 +10322,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="74" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>299</v>
       </c>
@@ -10800,7 +10800,7 @@
     </row>
     <row r="90" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
     <row r="91" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="92" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>342</v>
       </c>
@@ -10853,7 +10853,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="93" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>349</v>
       </c>
@@ -10880,7 +10880,7 @@
       </c>
     </row>
     <row r="94" spans="1:27" hidden="1" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>352</v>
       </c>
@@ -10927,7 +10927,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="96" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>356</v>
       </c>
@@ -10947,7 +10947,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="97" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>358</v>
       </c>
@@ -10967,7 +10967,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="98" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:27" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>360</v>
       </c>

</xml_diff>